<commit_message>
docs(project): align received hardware records
</commit_message>
<xml_diff>
--- a/docs/project/BOM.xlsx
+++ b/docs/project/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joeroche/Documents/excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gcecnjorg-my.sharepoint.com/personal/roche_joseph_students_gcecnj_org/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EA2F4A5C-250F-BA49-B4DC-FB62BCA7F71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C74FFC4-4AE3-4088-8329-AA132B53BCFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1300" yWindow="660" windowWidth="28100" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1220" yWindow="660" windowWidth="28180" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -366,10 +366,10 @@
     <t>Strawberry Pets Store</t>
   </si>
   <si>
-    <t>MR115ZZ Flanged Ball Bearing (10pcs)</t>
-  </si>
-  <si>
-    <t>5x11x4mm MR115ZZ flanged 10pcs</t>
+    <t>MR85ZZ Ball Bearing (10pcs)</t>
+  </si>
+  <si>
+    <t>5x8x2.5mm MR85RS 10pcs blue seals</t>
   </si>
   <si>
     <t>8210696713585240</t>
@@ -381,7 +381,7 @@
     <t>Neoprene Rubber Gasket Strip</t>
   </si>
   <si>
-    <t>2000x19x3mm neoprene belt strip target</t>
+    <t>2000x15x3mm anti-vibration neoprene</t>
   </si>
   <si>
     <t>8210696713565240</t>
@@ -390,7 +390,7 @@
     <t>U Officer Store</t>
   </si>
   <si>
-    <t>2000x19x3mm neoprene belt strip backup</t>
+    <t>2000x25x3mm anti-vibration neoprene</t>
   </si>
   <si>
     <t>8210696713545240</t>
@@ -886,7 +886,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -899,41 +899,35 @@
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1021,7 +1015,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1034,6 +1027,7 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1337,7 +1331,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="3" width="14" customWidth="1"/>
@@ -1345,17 +1339,17 @@
     <col min="6" max="6" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:6" ht="27.95" customHeight="1">
+      <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-    </row>
-    <row r="2" spans="1:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+    </row>
+    <row r="2" spans="1:6" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1375,7 +1369,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="18" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1395,7 +1389,7 @@
         <v>149.52000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="18" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
@@ -1415,7 +1409,7 @@
         <v>174.5</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="18" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
@@ -1435,14 +1429,14 @@
         <v>62.87</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="22" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="21.95" customHeight="1">
       <c r="A6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
       <c r="F6" s="4">
         <v>386.89</v>
       </c>
@@ -1459,7 +1453,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="38" customWidth="1"/>
@@ -1474,25 +1468,25 @@
     <col min="14" max="14" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:14" ht="27.95" customHeight="1">
+      <c r="A1" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="11"/>
-      <c r="M1" s="11"/>
-      <c r="N1" s="11"/>
-    </row>
-    <row r="2" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
+    </row>
+    <row r="2" spans="1:14" ht="24" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -1536,7 +1530,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" ht="26.1" customHeight="1">
       <c r="A3" s="5">
         <v>1</v>
       </c>
@@ -1580,7 +1574,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="26.1" customHeight="1">
       <c r="A4" s="5">
         <v>2</v>
       </c>
@@ -1624,7 +1618,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="26.1" customHeight="1">
       <c r="A5" s="5">
         <v>3</v>
       </c>
@@ -1668,7 +1662,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="26.1" customHeight="1">
       <c r="A6" s="5">
         <v>4</v>
       </c>
@@ -1712,7 +1706,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="26.1" customHeight="1">
       <c r="A7" s="5">
         <v>5</v>
       </c>
@@ -1756,7 +1750,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="26.1" customHeight="1">
       <c r="A8" s="5">
         <v>6</v>
       </c>
@@ -1800,7 +1794,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="26.1" customHeight="1">
       <c r="A9" s="5">
         <v>7</v>
       </c>
@@ -1844,7 +1838,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="26.1" customHeight="1">
       <c r="A10" s="5">
         <v>8</v>
       </c>
@@ -1888,7 +1882,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="26.1" customHeight="1">
       <c r="A11" s="5">
         <v>9</v>
       </c>
@@ -1932,7 +1926,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="26.1" customHeight="1">
       <c r="A12" s="5">
         <v>10</v>
       </c>
@@ -1976,7 +1970,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="26.1" customHeight="1">
       <c r="A13" s="5">
         <v>11</v>
       </c>
@@ -2020,7 +2014,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="26.1" customHeight="1">
       <c r="A14" s="5">
         <v>12</v>
       </c>
@@ -2064,7 +2058,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="26.1" customHeight="1">
       <c r="A15" s="5">
         <v>13</v>
       </c>
@@ -2108,7 +2102,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="26.1" customHeight="1">
       <c r="A16" s="5">
         <v>14</v>
       </c>
@@ -2152,7 +2146,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="26.1" customHeight="1">
       <c r="A17" s="5">
         <v>15</v>
       </c>
@@ -2196,7 +2190,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" ht="26.1" customHeight="1">
       <c r="A18" s="5">
         <v>16</v>
       </c>
@@ -2240,7 +2234,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="26.1" customHeight="1">
       <c r="A19" s="5">
         <v>17</v>
       </c>
@@ -2284,7 +2278,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" ht="26.1" customHeight="1">
       <c r="A20" s="5">
         <v>18</v>
       </c>
@@ -2328,7 +2322,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="26.1" customHeight="1">
       <c r="A21" s="5">
         <v>19</v>
       </c>
@@ -2372,7 +2366,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="26.1" customHeight="1">
       <c r="A22" s="5">
         <v>20</v>
       </c>
@@ -2416,7 +2410,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="26.1" customHeight="1">
       <c r="A23" s="5">
         <v>21</v>
       </c>
@@ -2460,7 +2454,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="26.1" customHeight="1">
       <c r="A24" s="5">
         <v>22</v>
       </c>
@@ -2504,7 +2498,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="26.1" customHeight="1">
       <c r="A25" s="5">
         <v>23</v>
       </c>
@@ -2548,7 +2542,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="26.1" customHeight="1">
       <c r="A26" s="5">
         <v>24</v>
       </c>
@@ -2592,7 +2586,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="26.1" customHeight="1">
       <c r="A27" s="5">
         <v>25</v>
       </c>
@@ -2636,7 +2630,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" ht="26.1" customHeight="1">
       <c r="A28" s="5">
         <v>26</v>
       </c>
@@ -2680,7 +2674,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" ht="26.1" customHeight="1">
       <c r="A29" s="5">
         <v>27</v>
       </c>
@@ -2724,7 +2718,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="26.1" customHeight="1">
       <c r="A30" s="5">
         <v>28</v>
       </c>
@@ -2768,7 +2762,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="26.1" customHeight="1">
       <c r="A31" s="5">
         <v>29</v>
       </c>
@@ -2812,7 +2806,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="26.1" customHeight="1">
       <c r="A32" s="5">
         <v>30</v>
       </c>
@@ -2856,7 +2850,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" ht="26.1" customHeight="1">
       <c r="A33" s="5">
         <v>31</v>
       </c>
@@ -2900,7 +2894,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" ht="26.1" customHeight="1">
       <c r="A34" s="5">
         <v>32</v>
       </c>
@@ -2944,7 +2938,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" ht="26.1" customHeight="1">
       <c r="A35" s="5">
         <v>33</v>
       </c>
@@ -2988,7 +2982,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" ht="26.1" customHeight="1">
       <c r="A36" s="5">
         <v>34</v>
       </c>
@@ -3032,7 +3026,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" ht="26.1" customHeight="1">
       <c r="A37" s="5">
         <v>35</v>
       </c>
@@ -3076,7 +3070,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" ht="26.1" customHeight="1">
       <c r="A38" s="5">
         <v>36</v>
       </c>
@@ -3120,17 +3114,17 @@
         <v>159</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="13" t="s">
+    <row r="39" spans="1:14" ht="20.100000000000001" customHeight="1">
+      <c r="A39" s="12" t="s">
         <v>162</v>
       </c>
-      <c r="B39" s="11"/>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="11"/>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
+      <c r="H39" s="15"/>
       <c r="I39" s="6">
         <v>340.33</v>
       </c>
@@ -3158,7 +3152,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I163"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
@@ -3171,20 +3165,20 @@
     <col min="9" max="9" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:9" ht="27.95" customHeight="1">
+      <c r="A1" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-    </row>
-    <row r="2" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+    </row>
+    <row r="2" spans="1:9" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
@@ -3213,7 +3207,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="24" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>49</v>
       </c>
@@ -3242,67 +3236,67 @@
         <v>18.03</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:9" ht="15" customHeight="1">
+      <c r="A4" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
       <c r="I4" s="8">
         <v>18.03</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+    <row r="5" spans="1:9" ht="15" customHeight="1">
+      <c r="A5" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
       <c r="I5" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:9" ht="15" customHeight="1">
+      <c r="A6" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="11"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
       <c r="I6" s="8">
         <v>1.19</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="13" t="s">
+    <row r="7" spans="1:9" ht="18" customHeight="1">
+      <c r="A7" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="11"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
+      <c r="G7" s="15"/>
+      <c r="H7" s="15"/>
       <c r="I7" s="6">
         <v>19.22</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" ht="24" customHeight="1">
       <c r="A9" s="2" t="s">
         <v>54</v>
       </c>
@@ -3331,67 +3325,67 @@
         <v>15.09</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="14" t="s">
+    <row r="10" spans="1:9" ht="15" customHeight="1">
+      <c r="A10" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
       <c r="I10" s="8">
         <v>15.09</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="14" t="s">
+    <row r="11" spans="1:9" ht="15" customHeight="1">
+      <c r="A11" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="15"/>
+      <c r="H11" s="15"/>
       <c r="I11" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="14" t="s">
+    <row r="12" spans="1:9" ht="15" customHeight="1">
+      <c r="A12" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="11"/>
-      <c r="E12" s="11"/>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="11"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
       <c r="I12" s="8">
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="13" t="s">
+    <row r="13" spans="1:9" ht="18" customHeight="1">
+      <c r="A13" s="12" t="s">
         <v>173</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="11"/>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
+      <c r="H13" s="15"/>
       <c r="I13" s="6">
         <v>16.23</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" ht="24" customHeight="1">
       <c r="A15" s="2" t="s">
         <v>58</v>
       </c>
@@ -3420,67 +3414,67 @@
         <v>11.66</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="14" t="s">
+    <row r="16" spans="1:9" ht="15" customHeight="1">
+      <c r="A16" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
       <c r="I16" s="8">
         <v>11.66</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="14" t="s">
+    <row r="17" spans="1:9" ht="15" customHeight="1">
+      <c r="A17" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15"/>
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+      <c r="H17" s="15"/>
       <c r="I17" s="8">
         <v>8.27</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="14" t="s">
+    <row r="18" spans="1:9" ht="15" customHeight="1">
+      <c r="A18" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="15"/>
+      <c r="H18" s="15"/>
       <c r="I18" s="8">
         <v>1.32</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:9" ht="18" customHeight="1">
+      <c r="A19" s="12" t="s">
         <v>177</v>
       </c>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
+      <c r="B19" s="15"/>
+      <c r="C19" s="15"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="15"/>
+      <c r="H19" s="15"/>
       <c r="I19" s="6">
         <v>21.25</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" ht="24" customHeight="1">
       <c r="A21" s="2" t="s">
         <v>62</v>
       </c>
@@ -3509,67 +3503,67 @@
         <v>0.79</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="14" t="s">
+    <row r="22" spans="1:9" ht="15" customHeight="1">
+      <c r="A22" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11"/>
-      <c r="E22" s="11"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15"/>
+      <c r="D22" s="15"/>
+      <c r="E22" s="15"/>
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
       <c r="I22" s="8">
         <v>0.79</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="14" t="s">
+    <row r="23" spans="1:9" ht="15" customHeight="1">
+      <c r="A23" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11"/>
-      <c r="E23" s="11"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="11"/>
-      <c r="H23" s="11"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+      <c r="G23" s="15"/>
+      <c r="H23" s="15"/>
       <c r="I23" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="14" t="s">
+    <row r="24" spans="1:9" ht="15" customHeight="1">
+      <c r="A24" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="11"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="11"/>
-      <c r="H24" s="11"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
       <c r="I24" s="8">
         <v>0.05</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:9" ht="18" customHeight="1">
+      <c r="A25" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="G25" s="11"/>
-      <c r="H25" s="11"/>
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="G25" s="15"/>
+      <c r="H25" s="15"/>
       <c r="I25" s="6">
         <v>0.84</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" ht="24" customHeight="1">
       <c r="A27" s="2" t="s">
         <v>66</v>
       </c>
@@ -3598,67 +3592,67 @@
         <v>1.46</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="14" t="s">
+    <row r="28" spans="1:9" ht="15" customHeight="1">
+      <c r="A28" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="B28" s="11"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="11"/>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15"/>
+      <c r="H28" s="15"/>
       <c r="I28" s="8">
         <v>1.46</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="14" t="s">
+    <row r="29" spans="1:9" ht="15" customHeight="1">
+      <c r="A29" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="B29" s="11"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="11"/>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
       <c r="I29" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="14" t="s">
+    <row r="30" spans="1:9" ht="15" customHeight="1">
+      <c r="A30" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="B30" s="11"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="11"/>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15"/>
+      <c r="H30" s="15"/>
       <c r="I30" s="8">
         <v>0.1</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="13" t="s">
+    <row r="31" spans="1:9" ht="18" customHeight="1">
+      <c r="A31" s="12" t="s">
         <v>185</v>
       </c>
-      <c r="B31" s="11"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="11"/>
-      <c r="E31" s="11"/>
-      <c r="F31" s="11"/>
-      <c r="G31" s="11"/>
-      <c r="H31" s="11"/>
+      <c r="B31" s="15"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15"/>
+      <c r="H31" s="15"/>
       <c r="I31" s="6">
         <v>1.56</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" ht="24" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>71</v>
       </c>
@@ -3687,67 +3681,67 @@
         <v>2.76</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="14" t="s">
+    <row r="34" spans="1:9" ht="15" customHeight="1">
+      <c r="A34" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="B34" s="11"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="11"/>
-      <c r="F34" s="11"/>
-      <c r="G34" s="11"/>
-      <c r="H34" s="11"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
       <c r="I34" s="8">
         <v>2.76</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="14" t="s">
+    <row r="35" spans="1:9" ht="15" customHeight="1">
+      <c r="A35" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="11"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="11"/>
-      <c r="H35" s="11"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
       <c r="I35" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="14" t="s">
+    <row r="36" spans="1:9" ht="15" customHeight="1">
+      <c r="A36" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="B36" s="11"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="11"/>
-      <c r="E36" s="11"/>
-      <c r="F36" s="11"/>
-      <c r="G36" s="11"/>
-      <c r="H36" s="11"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
       <c r="I36" s="8">
         <v>0.18</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="13" t="s">
+    <row r="37" spans="1:9" ht="18" customHeight="1">
+      <c r="A37" s="12" t="s">
         <v>189</v>
       </c>
-      <c r="B37" s="11"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="11"/>
-      <c r="F37" s="11"/>
-      <c r="G37" s="11"/>
-      <c r="H37" s="11"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15"/>
+      <c r="H37" s="15"/>
       <c r="I37" s="6">
         <v>2.94</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" ht="24" customHeight="1">
       <c r="A39" s="2" t="s">
         <v>74</v>
       </c>
@@ -3776,7 +3770,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" ht="24" customHeight="1">
       <c r="A40" s="2" t="s">
         <v>74</v>
       </c>
@@ -3805,67 +3799,67 @@
         <v>3.73</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="14" t="s">
+    <row r="41" spans="1:9" ht="15" customHeight="1">
+      <c r="A41" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
-      <c r="F41" s="11"/>
-      <c r="G41" s="11"/>
-      <c r="H41" s="11"/>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15"/>
+      <c r="D41" s="15"/>
+      <c r="E41" s="15"/>
+      <c r="F41" s="15"/>
+      <c r="G41" s="15"/>
+      <c r="H41" s="15"/>
       <c r="I41" s="8">
         <v>6.73</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="14" t="s">
+    <row r="42" spans="1:9" ht="15" customHeight="1">
+      <c r="A42" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="B42" s="11"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="11"/>
-      <c r="F42" s="11"/>
-      <c r="G42" s="11"/>
-      <c r="H42" s="11"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="15"/>
+      <c r="D42" s="15"/>
+      <c r="E42" s="15"/>
+      <c r="F42" s="15"/>
+      <c r="G42" s="15"/>
+      <c r="H42" s="15"/>
       <c r="I42" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="14" t="s">
+    <row r="43" spans="1:9" ht="15" customHeight="1">
+      <c r="A43" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="B43" s="11"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="11"/>
-      <c r="F43" s="11"/>
-      <c r="G43" s="11"/>
-      <c r="H43" s="11"/>
+      <c r="B43" s="15"/>
+      <c r="C43" s="15"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="15"/>
+      <c r="G43" s="15"/>
+      <c r="H43" s="15"/>
       <c r="I43" s="8">
         <v>0.45</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="13" t="s">
+    <row r="44" spans="1:9" ht="18" customHeight="1">
+      <c r="A44" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="B44" s="11"/>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="11"/>
-      <c r="F44" s="11"/>
-      <c r="G44" s="11"/>
-      <c r="H44" s="11"/>
+      <c r="B44" s="15"/>
+      <c r="C44" s="15"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="15"/>
+      <c r="F44" s="15"/>
+      <c r="G44" s="15"/>
+      <c r="H44" s="15"/>
       <c r="I44" s="6">
         <v>7.18</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" ht="24" customHeight="1">
       <c r="A46" s="2" t="s">
         <v>78</v>
       </c>
@@ -3894,67 +3888,67 @@
         <v>1.97</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="14" t="s">
+    <row r="47" spans="1:9" ht="15" customHeight="1">
+      <c r="A47" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="B47" s="11"/>
-      <c r="C47" s="11"/>
-      <c r="D47" s="11"/>
-      <c r="E47" s="11"/>
-      <c r="F47" s="11"/>
-      <c r="G47" s="11"/>
-      <c r="H47" s="11"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="15"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="15"/>
+      <c r="G47" s="15"/>
+      <c r="H47" s="15"/>
       <c r="I47" s="8">
         <v>1.97</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="14" t="s">
+    <row r="48" spans="1:9" ht="15" customHeight="1">
+      <c r="A48" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-      <c r="G48" s="11"/>
-      <c r="H48" s="11"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
+      <c r="H48" s="15"/>
       <c r="I48" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="14" t="s">
+    <row r="49" spans="1:9" ht="15" customHeight="1">
+      <c r="A49" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="B49" s="11"/>
-      <c r="C49" s="11"/>
-      <c r="D49" s="11"/>
-      <c r="E49" s="11"/>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
+      <c r="B49" s="15"/>
+      <c r="C49" s="15"/>
+      <c r="D49" s="15"/>
+      <c r="E49" s="15"/>
+      <c r="F49" s="15"/>
+      <c r="G49" s="15"/>
+      <c r="H49" s="15"/>
       <c r="I49" s="8">
         <v>0.13</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="13" t="s">
+    <row r="50" spans="1:9" ht="18" customHeight="1">
+      <c r="A50" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="B50" s="11"/>
-      <c r="C50" s="11"/>
-      <c r="D50" s="11"/>
-      <c r="E50" s="11"/>
-      <c r="F50" s="11"/>
-      <c r="G50" s="11"/>
-      <c r="H50" s="11"/>
+      <c r="B50" s="15"/>
+      <c r="C50" s="15"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="15"/>
+      <c r="G50" s="15"/>
+      <c r="H50" s="15"/>
       <c r="I50" s="6">
         <v>2.1</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" ht="24" customHeight="1">
       <c r="A52" s="2" t="s">
         <v>82</v>
       </c>
@@ -3983,67 +3977,67 @@
         <v>4.93</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="14" t="s">
+    <row r="53" spans="1:9" ht="15" customHeight="1">
+      <c r="A53" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="B53" s="11"/>
-      <c r="C53" s="11"/>
-      <c r="D53" s="11"/>
-      <c r="E53" s="11"/>
-      <c r="F53" s="11"/>
-      <c r="G53" s="11"/>
-      <c r="H53" s="11"/>
+      <c r="B53" s="15"/>
+      <c r="C53" s="15"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="15"/>
+      <c r="H53" s="15"/>
       <c r="I53" s="8">
         <v>4.93</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="14" t="s">
+    <row r="54" spans="1:9" ht="15" customHeight="1">
+      <c r="A54" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="11"/>
-      <c r="H54" s="11"/>
+      <c r="B54" s="15"/>
+      <c r="C54" s="15"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="15"/>
+      <c r="H54" s="15"/>
       <c r="I54" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="14" t="s">
+    <row r="55" spans="1:9" ht="15" customHeight="1">
+      <c r="A55" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="B55" s="11"/>
-      <c r="C55" s="11"/>
-      <c r="D55" s="11"/>
-      <c r="E55" s="11"/>
-      <c r="F55" s="11"/>
-      <c r="G55" s="11"/>
-      <c r="H55" s="11"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="15"/>
       <c r="I55" s="8">
         <v>0.33</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="13" t="s">
+    <row r="56" spans="1:9" ht="18" customHeight="1">
+      <c r="A56" s="12" t="s">
         <v>201</v>
       </c>
-      <c r="B56" s="11"/>
-      <c r="C56" s="11"/>
-      <c r="D56" s="11"/>
-      <c r="E56" s="11"/>
-      <c r="F56" s="11"/>
-      <c r="G56" s="11"/>
-      <c r="H56" s="11"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="15"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="15"/>
+      <c r="H56" s="15"/>
       <c r="I56" s="6">
         <v>5.26</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9" ht="24" customHeight="1">
       <c r="A58" s="2" t="s">
         <v>86</v>
       </c>
@@ -4072,67 +4066,67 @@
         <v>3.09</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="14" t="s">
+    <row r="59" spans="1:9" ht="15" customHeight="1">
+      <c r="A59" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="B59" s="11"/>
-      <c r="C59" s="11"/>
-      <c r="D59" s="11"/>
-      <c r="E59" s="11"/>
-      <c r="F59" s="11"/>
-      <c r="G59" s="11"/>
-      <c r="H59" s="11"/>
+      <c r="B59" s="15"/>
+      <c r="C59" s="15"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="15"/>
+      <c r="G59" s="15"/>
+      <c r="H59" s="15"/>
       <c r="I59" s="8">
         <v>3.09</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="14" t="s">
+    <row r="60" spans="1:9" ht="15" customHeight="1">
+      <c r="A60" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="B60" s="11"/>
-      <c r="C60" s="11"/>
-      <c r="D60" s="11"/>
-      <c r="E60" s="11"/>
-      <c r="F60" s="11"/>
-      <c r="G60" s="11"/>
-      <c r="H60" s="11"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
       <c r="I60" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="14" t="s">
+    <row r="61" spans="1:9" ht="15" customHeight="1">
+      <c r="A61" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
-      <c r="F61" s="11"/>
-      <c r="G61" s="11"/>
-      <c r="H61" s="11"/>
+      <c r="B61" s="15"/>
+      <c r="C61" s="15"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="15"/>
+      <c r="G61" s="15"/>
+      <c r="H61" s="15"/>
       <c r="I61" s="8">
         <v>0.2</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="13" t="s">
+    <row r="62" spans="1:9" ht="18" customHeight="1">
+      <c r="A62" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="B62" s="11"/>
-      <c r="C62" s="11"/>
-      <c r="D62" s="11"/>
-      <c r="E62" s="11"/>
-      <c r="F62" s="11"/>
-      <c r="G62" s="11"/>
-      <c r="H62" s="11"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="15"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="15"/>
+      <c r="H62" s="15"/>
       <c r="I62" s="6">
         <v>3.29</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:9" ht="24" customHeight="1">
       <c r="A64" s="2" t="s">
         <v>90</v>
       </c>
@@ -4161,67 +4155,67 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="14" t="s">
+    <row r="65" spans="1:9" ht="15" customHeight="1">
+      <c r="A65" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="B65" s="11"/>
-      <c r="C65" s="11"/>
-      <c r="D65" s="11"/>
-      <c r="E65" s="11"/>
-      <c r="F65" s="11"/>
-      <c r="G65" s="11"/>
-      <c r="H65" s="11"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="15"/>
+      <c r="H65" s="15"/>
       <c r="I65" s="8">
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="14" t="s">
+    <row r="66" spans="1:9" ht="15" customHeight="1">
+      <c r="A66" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="B66" s="11"/>
-      <c r="C66" s="11"/>
-      <c r="D66" s="11"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="11"/>
-      <c r="G66" s="11"/>
-      <c r="H66" s="11"/>
+      <c r="B66" s="15"/>
+      <c r="C66" s="15"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15"/>
+      <c r="F66" s="15"/>
+      <c r="G66" s="15"/>
+      <c r="H66" s="15"/>
       <c r="I66" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="14" t="s">
+    <row r="67" spans="1:9" ht="15" customHeight="1">
+      <c r="A67" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="B67" s="11"/>
-      <c r="C67" s="11"/>
-      <c r="D67" s="11"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="11"/>
-      <c r="G67" s="11"/>
-      <c r="H67" s="11"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="15"/>
+      <c r="D67" s="15"/>
+      <c r="E67" s="15"/>
+      <c r="F67" s="15"/>
+      <c r="G67" s="15"/>
+      <c r="H67" s="15"/>
       <c r="I67" s="8">
         <v>0.15</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="13" t="s">
+    <row r="68" spans="1:9" ht="18" customHeight="1">
+      <c r="A68" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="B68" s="11"/>
-      <c r="C68" s="11"/>
-      <c r="D68" s="11"/>
-      <c r="E68" s="11"/>
-      <c r="F68" s="11"/>
-      <c r="G68" s="11"/>
-      <c r="H68" s="11"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="15"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="15"/>
+      <c r="F68" s="15"/>
+      <c r="G68" s="15"/>
+      <c r="H68" s="15"/>
       <c r="I68" s="6">
         <v>2.39</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9" ht="24" customHeight="1">
       <c r="A70" s="2" t="s">
         <v>94</v>
       </c>
@@ -4250,67 +4244,67 @@
         <v>2.21</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="14" t="s">
+    <row r="71" spans="1:9" ht="15" customHeight="1">
+      <c r="A71" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="B71" s="11"/>
-      <c r="C71" s="11"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="11"/>
-      <c r="F71" s="11"/>
-      <c r="G71" s="11"/>
-      <c r="H71" s="11"/>
+      <c r="B71" s="15"/>
+      <c r="C71" s="15"/>
+      <c r="D71" s="15"/>
+      <c r="E71" s="15"/>
+      <c r="F71" s="15"/>
+      <c r="G71" s="15"/>
+      <c r="H71" s="15"/>
       <c r="I71" s="8">
         <v>2.21</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="14" t="s">
+    <row r="72" spans="1:9" ht="15" customHeight="1">
+      <c r="A72" s="13" t="s">
         <v>211</v>
       </c>
-      <c r="B72" s="11"/>
-      <c r="C72" s="11"/>
-      <c r="D72" s="11"/>
-      <c r="E72" s="11"/>
-      <c r="F72" s="11"/>
-      <c r="G72" s="11"/>
-      <c r="H72" s="11"/>
+      <c r="B72" s="15"/>
+      <c r="C72" s="15"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="15"/>
+      <c r="F72" s="15"/>
+      <c r="G72" s="15"/>
+      <c r="H72" s="15"/>
       <c r="I72" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="14" t="s">
+    <row r="73" spans="1:9" ht="15" customHeight="1">
+      <c r="A73" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="B73" s="11"/>
-      <c r="C73" s="11"/>
-      <c r="D73" s="11"/>
-      <c r="E73" s="11"/>
-      <c r="F73" s="11"/>
-      <c r="G73" s="11"/>
-      <c r="H73" s="11"/>
+      <c r="B73" s="15"/>
+      <c r="C73" s="15"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15"/>
+      <c r="F73" s="15"/>
+      <c r="G73" s="15"/>
+      <c r="H73" s="15"/>
       <c r="I73" s="8">
         <v>0.15</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="13" t="s">
+    <row r="74" spans="1:9" ht="18" customHeight="1">
+      <c r="A74" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="B74" s="11"/>
-      <c r="C74" s="11"/>
-      <c r="D74" s="11"/>
-      <c r="E74" s="11"/>
-      <c r="F74" s="11"/>
-      <c r="G74" s="11"/>
-      <c r="H74" s="11"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="15"/>
+      <c r="D74" s="15"/>
+      <c r="E74" s="15"/>
+      <c r="F74" s="15"/>
+      <c r="G74" s="15"/>
+      <c r="H74" s="15"/>
       <c r="I74" s="6">
         <v>2.36</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9" ht="24" customHeight="1">
       <c r="A76" s="2" t="s">
         <v>98</v>
       </c>
@@ -4339,67 +4333,67 @@
         <v>1.89</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="14" t="s">
+    <row r="77" spans="1:9" ht="15" customHeight="1">
+      <c r="A77" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="B77" s="11"/>
-      <c r="C77" s="11"/>
-      <c r="D77" s="11"/>
-      <c r="E77" s="11"/>
-      <c r="F77" s="11"/>
-      <c r="G77" s="11"/>
-      <c r="H77" s="11"/>
+      <c r="B77" s="15"/>
+      <c r="C77" s="15"/>
+      <c r="D77" s="15"/>
+      <c r="E77" s="15"/>
+      <c r="F77" s="15"/>
+      <c r="G77" s="15"/>
+      <c r="H77" s="15"/>
       <c r="I77" s="8">
         <v>1.89</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="14" t="s">
+    <row r="78" spans="1:9" ht="15" customHeight="1">
+      <c r="A78" s="13" t="s">
         <v>215</v>
       </c>
-      <c r="B78" s="11"/>
-      <c r="C78" s="11"/>
-      <c r="D78" s="11"/>
-      <c r="E78" s="11"/>
-      <c r="F78" s="11"/>
-      <c r="G78" s="11"/>
-      <c r="H78" s="11"/>
+      <c r="B78" s="15"/>
+      <c r="C78" s="15"/>
+      <c r="D78" s="15"/>
+      <c r="E78" s="15"/>
+      <c r="F78" s="15"/>
+      <c r="G78" s="15"/>
+      <c r="H78" s="15"/>
       <c r="I78" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="14" t="s">
+    <row r="79" spans="1:9" ht="15" customHeight="1">
+      <c r="A79" s="13" t="s">
         <v>216</v>
       </c>
-      <c r="B79" s="11"/>
-      <c r="C79" s="11"/>
-      <c r="D79" s="11"/>
-      <c r="E79" s="11"/>
-      <c r="F79" s="11"/>
-      <c r="G79" s="11"/>
-      <c r="H79" s="11"/>
+      <c r="B79" s="15"/>
+      <c r="C79" s="15"/>
+      <c r="D79" s="15"/>
+      <c r="E79" s="15"/>
+      <c r="F79" s="15"/>
+      <c r="G79" s="15"/>
+      <c r="H79" s="15"/>
       <c r="I79" s="8">
         <v>0.13</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="13" t="s">
+    <row r="80" spans="1:9" ht="18" customHeight="1">
+      <c r="A80" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="B80" s="11"/>
-      <c r="C80" s="11"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="11"/>
-      <c r="F80" s="11"/>
-      <c r="G80" s="11"/>
-      <c r="H80" s="11"/>
+      <c r="B80" s="15"/>
+      <c r="C80" s="15"/>
+      <c r="D80" s="15"/>
+      <c r="E80" s="15"/>
+      <c r="F80" s="15"/>
+      <c r="G80" s="15"/>
+      <c r="H80" s="15"/>
       <c r="I80" s="6">
         <v>2.02</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:9" ht="24" customHeight="1">
       <c r="A82" s="2" t="s">
         <v>102</v>
       </c>
@@ -4428,67 +4422,67 @@
         <v>10.14</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="14" t="s">
+    <row r="83" spans="1:9" ht="15" customHeight="1">
+      <c r="A83" s="13" t="s">
         <v>218</v>
       </c>
-      <c r="B83" s="11"/>
-      <c r="C83" s="11"/>
-      <c r="D83" s="11"/>
-      <c r="E83" s="11"/>
-      <c r="F83" s="11"/>
-      <c r="G83" s="11"/>
-      <c r="H83" s="11"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="15"/>
+      <c r="D83" s="15"/>
+      <c r="E83" s="15"/>
+      <c r="F83" s="15"/>
+      <c r="G83" s="15"/>
+      <c r="H83" s="15"/>
       <c r="I83" s="8">
         <v>10.14</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="14" t="s">
+    <row r="84" spans="1:9" ht="15" customHeight="1">
+      <c r="A84" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="B84" s="11"/>
-      <c r="C84" s="11"/>
-      <c r="D84" s="11"/>
-      <c r="E84" s="11"/>
-      <c r="F84" s="11"/>
-      <c r="G84" s="11"/>
-      <c r="H84" s="11"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="15"/>
+      <c r="D84" s="15"/>
+      <c r="E84" s="15"/>
+      <c r="F84" s="15"/>
+      <c r="G84" s="15"/>
+      <c r="H84" s="15"/>
       <c r="I84" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="14" t="s">
+    <row r="85" spans="1:9" ht="15" customHeight="1">
+      <c r="A85" s="13" t="s">
         <v>220</v>
       </c>
-      <c r="B85" s="11"/>
-      <c r="C85" s="11"/>
-      <c r="D85" s="11"/>
-      <c r="E85" s="11"/>
-      <c r="F85" s="11"/>
-      <c r="G85" s="11"/>
-      <c r="H85" s="11"/>
+      <c r="B85" s="15"/>
+      <c r="C85" s="15"/>
+      <c r="D85" s="15"/>
+      <c r="E85" s="15"/>
+      <c r="F85" s="15"/>
+      <c r="G85" s="15"/>
+      <c r="H85" s="15"/>
       <c r="I85" s="8">
         <v>0.67</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="13" t="s">
+    <row r="86" spans="1:9" ht="18" customHeight="1">
+      <c r="A86" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="B86" s="11"/>
-      <c r="C86" s="11"/>
-      <c r="D86" s="11"/>
-      <c r="E86" s="11"/>
-      <c r="F86" s="11"/>
-      <c r="G86" s="11"/>
-      <c r="H86" s="11"/>
+      <c r="B86" s="15"/>
+      <c r="C86" s="15"/>
+      <c r="D86" s="15"/>
+      <c r="E86" s="15"/>
+      <c r="F86" s="15"/>
+      <c r="G86" s="15"/>
+      <c r="H86" s="15"/>
       <c r="I86" s="6">
         <v>10.81</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:9" ht="24" customHeight="1">
       <c r="A88" s="2" t="s">
         <v>106</v>
       </c>
@@ -4517,67 +4511,67 @@
         <v>3.72</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="14" t="s">
+    <row r="89" spans="1:9" ht="15" customHeight="1">
+      <c r="A89" s="13" t="s">
         <v>222</v>
       </c>
-      <c r="B89" s="11"/>
-      <c r="C89" s="11"/>
-      <c r="D89" s="11"/>
-      <c r="E89" s="11"/>
-      <c r="F89" s="11"/>
-      <c r="G89" s="11"/>
-      <c r="H89" s="11"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="15"/>
+      <c r="D89" s="15"/>
+      <c r="E89" s="15"/>
+      <c r="F89" s="15"/>
+      <c r="G89" s="15"/>
+      <c r="H89" s="15"/>
       <c r="I89" s="8">
         <v>3.72</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="14" t="s">
+    <row r="90" spans="1:9" ht="15" customHeight="1">
+      <c r="A90" s="13" t="s">
         <v>223</v>
       </c>
-      <c r="B90" s="11"/>
-      <c r="C90" s="11"/>
-      <c r="D90" s="11"/>
-      <c r="E90" s="11"/>
-      <c r="F90" s="11"/>
-      <c r="G90" s="11"/>
-      <c r="H90" s="11"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="15"/>
+      <c r="D90" s="15"/>
+      <c r="E90" s="15"/>
+      <c r="F90" s="15"/>
+      <c r="G90" s="15"/>
+      <c r="H90" s="15"/>
       <c r="I90" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="14" t="s">
+    <row r="91" spans="1:9" ht="15" customHeight="1">
+      <c r="A91" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="B91" s="11"/>
-      <c r="C91" s="11"/>
-      <c r="D91" s="11"/>
-      <c r="E91" s="11"/>
-      <c r="F91" s="11"/>
-      <c r="G91" s="11"/>
-      <c r="H91" s="11"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="15"/>
+      <c r="D91" s="15"/>
+      <c r="E91" s="15"/>
+      <c r="F91" s="15"/>
+      <c r="G91" s="15"/>
+      <c r="H91" s="15"/>
       <c r="I91" s="8">
         <v>0.25</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="13" t="s">
+    <row r="92" spans="1:9" ht="18" customHeight="1">
+      <c r="A92" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="B92" s="11"/>
-      <c r="C92" s="11"/>
-      <c r="D92" s="11"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="11"/>
-      <c r="G92" s="11"/>
-      <c r="H92" s="11"/>
+      <c r="B92" s="15"/>
+      <c r="C92" s="15"/>
+      <c r="D92" s="15"/>
+      <c r="E92" s="15"/>
+      <c r="F92" s="15"/>
+      <c r="G92" s="15"/>
+      <c r="H92" s="15"/>
       <c r="I92" s="6">
         <v>3.97</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:9" ht="24" customHeight="1">
       <c r="A94" s="2" t="s">
         <v>110</v>
       </c>
@@ -4606,67 +4600,67 @@
         <v>6.47</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="14" t="s">
+    <row r="95" spans="1:9" ht="15" customHeight="1">
+      <c r="A95" s="13" t="s">
         <v>226</v>
       </c>
-      <c r="B95" s="11"/>
-      <c r="C95" s="11"/>
-      <c r="D95" s="11"/>
-      <c r="E95" s="11"/>
-      <c r="F95" s="11"/>
-      <c r="G95" s="11"/>
-      <c r="H95" s="11"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="15"/>
+      <c r="D95" s="15"/>
+      <c r="E95" s="15"/>
+      <c r="F95" s="15"/>
+      <c r="G95" s="15"/>
+      <c r="H95" s="15"/>
       <c r="I95" s="8">
         <v>6.47</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="14" t="s">
+    <row r="96" spans="1:9" ht="15" customHeight="1">
+      <c r="A96" s="13" t="s">
         <v>227</v>
       </c>
-      <c r="B96" s="11"/>
-      <c r="C96" s="11"/>
-      <c r="D96" s="11"/>
-      <c r="E96" s="11"/>
-      <c r="F96" s="11"/>
-      <c r="G96" s="11"/>
-      <c r="H96" s="11"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="15"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15"/>
+      <c r="F96" s="15"/>
+      <c r="G96" s="15"/>
+      <c r="H96" s="15"/>
       <c r="I96" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="14" t="s">
+    <row r="97" spans="1:9" ht="15" customHeight="1">
+      <c r="A97" s="13" t="s">
         <v>228</v>
       </c>
-      <c r="B97" s="11"/>
-      <c r="C97" s="11"/>
-      <c r="D97" s="11"/>
-      <c r="E97" s="11"/>
-      <c r="F97" s="11"/>
-      <c r="G97" s="11"/>
-      <c r="H97" s="11"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="15"/>
+      <c r="D97" s="15"/>
+      <c r="E97" s="15"/>
+      <c r="F97" s="15"/>
+      <c r="G97" s="15"/>
+      <c r="H97" s="15"/>
       <c r="I97" s="8">
         <v>0.47</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="13" t="s">
+    <row r="98" spans="1:9" ht="18" customHeight="1">
+      <c r="A98" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="B98" s="11"/>
-      <c r="C98" s="11"/>
-      <c r="D98" s="11"/>
-      <c r="E98" s="11"/>
-      <c r="F98" s="11"/>
-      <c r="G98" s="11"/>
-      <c r="H98" s="11"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="15"/>
+      <c r="D98" s="15"/>
+      <c r="E98" s="15"/>
+      <c r="F98" s="15"/>
+      <c r="G98" s="15"/>
+      <c r="H98" s="15"/>
       <c r="I98" s="6">
         <v>6.94</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:9" ht="24" customHeight="1">
       <c r="A100" s="2" t="s">
         <v>114</v>
       </c>
@@ -4695,67 +4689,67 @@
         <v>4.68</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="14" t="s">
+    <row r="101" spans="1:9" ht="15" customHeight="1">
+      <c r="A101" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="B101" s="11"/>
-      <c r="C101" s="11"/>
-      <c r="D101" s="11"/>
-      <c r="E101" s="11"/>
-      <c r="F101" s="11"/>
-      <c r="G101" s="11"/>
-      <c r="H101" s="11"/>
+      <c r="B101" s="15"/>
+      <c r="C101" s="15"/>
+      <c r="D101" s="15"/>
+      <c r="E101" s="15"/>
+      <c r="F101" s="15"/>
+      <c r="G101" s="15"/>
+      <c r="H101" s="15"/>
       <c r="I101" s="8">
         <v>4.68</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="14" t="s">
+    <row r="102" spans="1:9" ht="15" customHeight="1">
+      <c r="A102" s="13" t="s">
         <v>231</v>
       </c>
-      <c r="B102" s="11"/>
-      <c r="C102" s="11"/>
-      <c r="D102" s="11"/>
-      <c r="E102" s="11"/>
-      <c r="F102" s="11"/>
-      <c r="G102" s="11"/>
-      <c r="H102" s="11"/>
+      <c r="B102" s="15"/>
+      <c r="C102" s="15"/>
+      <c r="D102" s="15"/>
+      <c r="E102" s="15"/>
+      <c r="F102" s="15"/>
+      <c r="G102" s="15"/>
+      <c r="H102" s="15"/>
       <c r="I102" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="14" t="s">
+    <row r="103" spans="1:9" ht="15" customHeight="1">
+      <c r="A103" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="B103" s="11"/>
-      <c r="C103" s="11"/>
-      <c r="D103" s="11"/>
-      <c r="E103" s="11"/>
-      <c r="F103" s="11"/>
-      <c r="G103" s="11"/>
-      <c r="H103" s="11"/>
+      <c r="B103" s="15"/>
+      <c r="C103" s="15"/>
+      <c r="D103" s="15"/>
+      <c r="E103" s="15"/>
+      <c r="F103" s="15"/>
+      <c r="G103" s="15"/>
+      <c r="H103" s="15"/>
       <c r="I103" s="8">
         <v>0.31</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="13" t="s">
+    <row r="104" spans="1:9" ht="18" customHeight="1">
+      <c r="A104" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="B104" s="11"/>
-      <c r="C104" s="11"/>
-      <c r="D104" s="11"/>
-      <c r="E104" s="11"/>
-      <c r="F104" s="11"/>
-      <c r="G104" s="11"/>
-      <c r="H104" s="11"/>
+      <c r="B104" s="15"/>
+      <c r="C104" s="15"/>
+      <c r="D104" s="15"/>
+      <c r="E104" s="15"/>
+      <c r="F104" s="15"/>
+      <c r="G104" s="15"/>
+      <c r="H104" s="15"/>
       <c r="I104" s="6">
         <v>4.99</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9" ht="24" customHeight="1">
       <c r="A106" s="2" t="s">
         <v>117</v>
       </c>
@@ -4784,67 +4778,67 @@
         <v>7.58</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="14" t="s">
+    <row r="107" spans="1:9" ht="15" customHeight="1">
+      <c r="A107" s="13" t="s">
         <v>234</v>
       </c>
-      <c r="B107" s="11"/>
-      <c r="C107" s="11"/>
-      <c r="D107" s="11"/>
-      <c r="E107" s="11"/>
-      <c r="F107" s="11"/>
-      <c r="G107" s="11"/>
-      <c r="H107" s="11"/>
+      <c r="B107" s="15"/>
+      <c r="C107" s="15"/>
+      <c r="D107" s="15"/>
+      <c r="E107" s="15"/>
+      <c r="F107" s="15"/>
+      <c r="G107" s="15"/>
+      <c r="H107" s="15"/>
       <c r="I107" s="8">
         <v>7.58</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="14" t="s">
+    <row r="108" spans="1:9" ht="15" customHeight="1">
+      <c r="A108" s="13" t="s">
         <v>235</v>
       </c>
-      <c r="B108" s="11"/>
-      <c r="C108" s="11"/>
-      <c r="D108" s="11"/>
-      <c r="E108" s="11"/>
-      <c r="F108" s="11"/>
-      <c r="G108" s="11"/>
-      <c r="H108" s="11"/>
+      <c r="B108" s="15"/>
+      <c r="C108" s="15"/>
+      <c r="D108" s="15"/>
+      <c r="E108" s="15"/>
+      <c r="F108" s="15"/>
+      <c r="G108" s="15"/>
+      <c r="H108" s="15"/>
       <c r="I108" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="14" t="s">
+    <row r="109" spans="1:9" ht="15" customHeight="1">
+      <c r="A109" s="13" t="s">
         <v>236</v>
       </c>
-      <c r="B109" s="11"/>
-      <c r="C109" s="11"/>
-      <c r="D109" s="11"/>
-      <c r="E109" s="11"/>
-      <c r="F109" s="11"/>
-      <c r="G109" s="11"/>
-      <c r="H109" s="11"/>
+      <c r="B109" s="15"/>
+      <c r="C109" s="15"/>
+      <c r="D109" s="15"/>
+      <c r="E109" s="15"/>
+      <c r="F109" s="15"/>
+      <c r="G109" s="15"/>
+      <c r="H109" s="15"/>
       <c r="I109" s="8">
         <v>0.5</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="13" t="s">
+    <row r="110" spans="1:9" ht="18" customHeight="1">
+      <c r="A110" s="12" t="s">
         <v>237</v>
       </c>
-      <c r="B110" s="11"/>
-      <c r="C110" s="11"/>
-      <c r="D110" s="11"/>
-      <c r="E110" s="11"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="11"/>
-      <c r="H110" s="11"/>
+      <c r="B110" s="15"/>
+      <c r="C110" s="15"/>
+      <c r="D110" s="15"/>
+      <c r="E110" s="15"/>
+      <c r="F110" s="15"/>
+      <c r="G110" s="15"/>
+      <c r="H110" s="15"/>
       <c r="I110" s="6">
         <v>8.08</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:9" ht="24" customHeight="1">
       <c r="A112" s="2" t="s">
         <v>120</v>
       </c>
@@ -4873,67 +4867,67 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="14" t="s">
+    <row r="113" spans="1:9" ht="15" customHeight="1">
+      <c r="A113" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="B113" s="11"/>
-      <c r="C113" s="11"/>
-      <c r="D113" s="11"/>
-      <c r="E113" s="11"/>
-      <c r="F113" s="11"/>
-      <c r="G113" s="11"/>
-      <c r="H113" s="11"/>
+      <c r="B113" s="15"/>
+      <c r="C113" s="15"/>
+      <c r="D113" s="15"/>
+      <c r="E113" s="15"/>
+      <c r="F113" s="15"/>
+      <c r="G113" s="15"/>
+      <c r="H113" s="15"/>
       <c r="I113" s="8">
         <v>1.44</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="14" t="s">
+    <row r="114" spans="1:9" ht="15" customHeight="1">
+      <c r="A114" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="B114" s="11"/>
-      <c r="C114" s="11"/>
-      <c r="D114" s="11"/>
-      <c r="E114" s="11"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="11"/>
-      <c r="H114" s="11"/>
+      <c r="B114" s="15"/>
+      <c r="C114" s="15"/>
+      <c r="D114" s="15"/>
+      <c r="E114" s="15"/>
+      <c r="F114" s="15"/>
+      <c r="G114" s="15"/>
+      <c r="H114" s="15"/>
       <c r="I114" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="14" t="s">
+    <row r="115" spans="1:9" ht="15" customHeight="1">
+      <c r="A115" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="B115" s="11"/>
-      <c r="C115" s="11"/>
-      <c r="D115" s="11"/>
-      <c r="E115" s="11"/>
-      <c r="F115" s="11"/>
-      <c r="G115" s="11"/>
-      <c r="H115" s="11"/>
+      <c r="B115" s="15"/>
+      <c r="C115" s="15"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="15"/>
+      <c r="F115" s="15"/>
+      <c r="G115" s="15"/>
+      <c r="H115" s="15"/>
       <c r="I115" s="8">
         <v>0.09</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="13" t="s">
+    <row r="116" spans="1:9" ht="18" customHeight="1">
+      <c r="A116" s="12" t="s">
         <v>241</v>
       </c>
-      <c r="B116" s="11"/>
-      <c r="C116" s="11"/>
-      <c r="D116" s="11"/>
-      <c r="E116" s="11"/>
-      <c r="F116" s="11"/>
-      <c r="G116" s="11"/>
-      <c r="H116" s="11"/>
+      <c r="B116" s="15"/>
+      <c r="C116" s="15"/>
+      <c r="D116" s="15"/>
+      <c r="E116" s="15"/>
+      <c r="F116" s="15"/>
+      <c r="G116" s="15"/>
+      <c r="H116" s="15"/>
       <c r="I116" s="6">
         <v>1.53</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:9" ht="24" customHeight="1">
       <c r="A118" s="2" t="s">
         <v>124</v>
       </c>
@@ -4962,67 +4956,67 @@
         <v>12.88</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="14" t="s">
+    <row r="119" spans="1:9" ht="15" customHeight="1">
+      <c r="A119" s="13" t="s">
         <v>242</v>
       </c>
-      <c r="B119" s="11"/>
-      <c r="C119" s="11"/>
-      <c r="D119" s="11"/>
-      <c r="E119" s="11"/>
-      <c r="F119" s="11"/>
-      <c r="G119" s="11"/>
-      <c r="H119" s="11"/>
+      <c r="B119" s="15"/>
+      <c r="C119" s="15"/>
+      <c r="D119" s="15"/>
+      <c r="E119" s="15"/>
+      <c r="F119" s="15"/>
+      <c r="G119" s="15"/>
+      <c r="H119" s="15"/>
       <c r="I119" s="8">
         <v>12.88</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="14" t="s">
+    <row r="120" spans="1:9" ht="15" customHeight="1">
+      <c r="A120" s="13" t="s">
         <v>243</v>
       </c>
-      <c r="B120" s="11"/>
-      <c r="C120" s="11"/>
-      <c r="D120" s="11"/>
-      <c r="E120" s="11"/>
-      <c r="F120" s="11"/>
-      <c r="G120" s="11"/>
-      <c r="H120" s="11"/>
+      <c r="B120" s="15"/>
+      <c r="C120" s="15"/>
+      <c r="D120" s="15"/>
+      <c r="E120" s="15"/>
+      <c r="F120" s="15"/>
+      <c r="G120" s="15"/>
+      <c r="H120" s="15"/>
       <c r="I120" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="14" t="s">
+    <row r="121" spans="1:9" ht="15" customHeight="1">
+      <c r="A121" s="13" t="s">
         <v>244</v>
       </c>
-      <c r="B121" s="11"/>
-      <c r="C121" s="11"/>
-      <c r="D121" s="11"/>
-      <c r="E121" s="11"/>
-      <c r="F121" s="11"/>
-      <c r="G121" s="11"/>
-      <c r="H121" s="11"/>
+      <c r="B121" s="15"/>
+      <c r="C121" s="15"/>
+      <c r="D121" s="15"/>
+      <c r="E121" s="15"/>
+      <c r="F121" s="15"/>
+      <c r="G121" s="15"/>
+      <c r="H121" s="15"/>
       <c r="I121" s="8">
         <v>0.93</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="13" t="s">
+    <row r="122" spans="1:9" ht="18" customHeight="1">
+      <c r="A122" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="B122" s="11"/>
-      <c r="C122" s="11"/>
-      <c r="D122" s="11"/>
-      <c r="E122" s="11"/>
-      <c r="F122" s="11"/>
-      <c r="G122" s="11"/>
-      <c r="H122" s="11"/>
+      <c r="B122" s="15"/>
+      <c r="C122" s="15"/>
+      <c r="D122" s="15"/>
+      <c r="E122" s="15"/>
+      <c r="F122" s="15"/>
+      <c r="G122" s="15"/>
+      <c r="H122" s="15"/>
       <c r="I122" s="6">
         <v>13.81</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:9" ht="24" customHeight="1">
       <c r="A124" s="2" t="s">
         <v>128</v>
       </c>
@@ -5051,67 +5045,67 @@
         <v>10.039999999999999</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="14" t="s">
+    <row r="125" spans="1:9" ht="15" customHeight="1">
+      <c r="A125" s="13" t="s">
         <v>246</v>
       </c>
-      <c r="B125" s="11"/>
-      <c r="C125" s="11"/>
-      <c r="D125" s="11"/>
-      <c r="E125" s="11"/>
-      <c r="F125" s="11"/>
-      <c r="G125" s="11"/>
-      <c r="H125" s="11"/>
+      <c r="B125" s="15"/>
+      <c r="C125" s="15"/>
+      <c r="D125" s="15"/>
+      <c r="E125" s="15"/>
+      <c r="F125" s="15"/>
+      <c r="G125" s="15"/>
+      <c r="H125" s="15"/>
       <c r="I125" s="8">
         <v>10.039999999999999</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A126" s="14" t="s">
+    <row r="126" spans="1:9" ht="15" customHeight="1">
+      <c r="A126" s="13" t="s">
         <v>247</v>
       </c>
-      <c r="B126" s="11"/>
-      <c r="C126" s="11"/>
-      <c r="D126" s="11"/>
-      <c r="E126" s="11"/>
-      <c r="F126" s="11"/>
-      <c r="G126" s="11"/>
-      <c r="H126" s="11"/>
+      <c r="B126" s="15"/>
+      <c r="C126" s="15"/>
+      <c r="D126" s="15"/>
+      <c r="E126" s="15"/>
+      <c r="F126" s="15"/>
+      <c r="G126" s="15"/>
+      <c r="H126" s="15"/>
       <c r="I126" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A127" s="14" t="s">
+    <row r="127" spans="1:9" ht="15" customHeight="1">
+      <c r="A127" s="13" t="s">
         <v>248</v>
       </c>
-      <c r="B127" s="11"/>
-      <c r="C127" s="11"/>
-      <c r="D127" s="11"/>
-      <c r="E127" s="11"/>
-      <c r="F127" s="11"/>
-      <c r="G127" s="11"/>
-      <c r="H127" s="11"/>
+      <c r="B127" s="15"/>
+      <c r="C127" s="15"/>
+      <c r="D127" s="15"/>
+      <c r="E127" s="15"/>
+      <c r="F127" s="15"/>
+      <c r="G127" s="15"/>
+      <c r="H127" s="15"/>
       <c r="I127" s="8">
         <v>0.67</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A128" s="13" t="s">
+    <row r="128" spans="1:9" ht="18" customHeight="1">
+      <c r="A128" s="12" t="s">
         <v>249</v>
       </c>
-      <c r="B128" s="11"/>
-      <c r="C128" s="11"/>
-      <c r="D128" s="11"/>
-      <c r="E128" s="11"/>
-      <c r="F128" s="11"/>
-      <c r="G128" s="11"/>
-      <c r="H128" s="11"/>
+      <c r="B128" s="15"/>
+      <c r="C128" s="15"/>
+      <c r="D128" s="15"/>
+      <c r="E128" s="15"/>
+      <c r="F128" s="15"/>
+      <c r="G128" s="15"/>
+      <c r="H128" s="15"/>
       <c r="I128" s="6">
         <v>10.71</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:9" ht="24" customHeight="1">
       <c r="A130" s="2" t="s">
         <v>132</v>
       </c>
@@ -5140,67 +5134,67 @@
         <v>4.5199999999999996</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A131" s="14" t="s">
+    <row r="131" spans="1:9" ht="15" customHeight="1">
+      <c r="A131" s="13" t="s">
         <v>250</v>
       </c>
-      <c r="B131" s="11"/>
-      <c r="C131" s="11"/>
-      <c r="D131" s="11"/>
-      <c r="E131" s="11"/>
-      <c r="F131" s="11"/>
-      <c r="G131" s="11"/>
-      <c r="H131" s="11"/>
+      <c r="B131" s="15"/>
+      <c r="C131" s="15"/>
+      <c r="D131" s="15"/>
+      <c r="E131" s="15"/>
+      <c r="F131" s="15"/>
+      <c r="G131" s="15"/>
+      <c r="H131" s="15"/>
       <c r="I131" s="8">
         <v>4.5199999999999996</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A132" s="14" t="s">
+    <row r="132" spans="1:9" ht="15" customHeight="1">
+      <c r="A132" s="13" t="s">
         <v>251</v>
       </c>
-      <c r="B132" s="11"/>
-      <c r="C132" s="11"/>
-      <c r="D132" s="11"/>
-      <c r="E132" s="11"/>
-      <c r="F132" s="11"/>
-      <c r="G132" s="11"/>
-      <c r="H132" s="11"/>
+      <c r="B132" s="15"/>
+      <c r="C132" s="15"/>
+      <c r="D132" s="15"/>
+      <c r="E132" s="15"/>
+      <c r="F132" s="15"/>
+      <c r="G132" s="15"/>
+      <c r="H132" s="15"/>
       <c r="I132" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A133" s="14" t="s">
+    <row r="133" spans="1:9" ht="15" customHeight="1">
+      <c r="A133" s="13" t="s">
         <v>252</v>
       </c>
-      <c r="B133" s="11"/>
-      <c r="C133" s="11"/>
-      <c r="D133" s="11"/>
-      <c r="E133" s="11"/>
-      <c r="F133" s="11"/>
-      <c r="G133" s="11"/>
-      <c r="H133" s="11"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="15"/>
+      <c r="D133" s="15"/>
+      <c r="E133" s="15"/>
+      <c r="F133" s="15"/>
+      <c r="G133" s="15"/>
+      <c r="H133" s="15"/>
       <c r="I133" s="8">
         <v>0.3</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A134" s="13" t="s">
+    <row r="134" spans="1:9" ht="18" customHeight="1">
+      <c r="A134" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="B134" s="11"/>
-      <c r="C134" s="11"/>
-      <c r="D134" s="11"/>
-      <c r="E134" s="11"/>
-      <c r="F134" s="11"/>
-      <c r="G134" s="11"/>
-      <c r="H134" s="11"/>
+      <c r="B134" s="15"/>
+      <c r="C134" s="15"/>
+      <c r="D134" s="15"/>
+      <c r="E134" s="15"/>
+      <c r="F134" s="15"/>
+      <c r="G134" s="15"/>
+      <c r="H134" s="15"/>
       <c r="I134" s="6">
         <v>4.82</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:9" ht="24" customHeight="1">
       <c r="A136" s="2" t="s">
         <v>136</v>
       </c>
@@ -5229,67 +5223,67 @@
         <v>1.69</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A137" s="14" t="s">
+    <row r="137" spans="1:9" ht="15" customHeight="1">
+      <c r="A137" s="13" t="s">
         <v>254</v>
       </c>
-      <c r="B137" s="11"/>
-      <c r="C137" s="11"/>
-      <c r="D137" s="11"/>
-      <c r="E137" s="11"/>
-      <c r="F137" s="11"/>
-      <c r="G137" s="11"/>
-      <c r="H137" s="11"/>
+      <c r="B137" s="15"/>
+      <c r="C137" s="15"/>
+      <c r="D137" s="15"/>
+      <c r="E137" s="15"/>
+      <c r="F137" s="15"/>
+      <c r="G137" s="15"/>
+      <c r="H137" s="15"/>
       <c r="I137" s="8">
         <v>1.69</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A138" s="14" t="s">
+    <row r="138" spans="1:9" ht="15" customHeight="1">
+      <c r="A138" s="13" t="s">
         <v>255</v>
       </c>
-      <c r="B138" s="11"/>
-      <c r="C138" s="11"/>
-      <c r="D138" s="11"/>
-      <c r="E138" s="11"/>
-      <c r="F138" s="11"/>
-      <c r="G138" s="11"/>
-      <c r="H138" s="11"/>
+      <c r="B138" s="15"/>
+      <c r="C138" s="15"/>
+      <c r="D138" s="15"/>
+      <c r="E138" s="15"/>
+      <c r="F138" s="15"/>
+      <c r="G138" s="15"/>
+      <c r="H138" s="15"/>
       <c r="I138" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A139" s="14" t="s">
+    <row r="139" spans="1:9" ht="15" customHeight="1">
+      <c r="A139" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="B139" s="11"/>
-      <c r="C139" s="11"/>
-      <c r="D139" s="11"/>
-      <c r="E139" s="11"/>
-      <c r="F139" s="11"/>
-      <c r="G139" s="11"/>
-      <c r="H139" s="11"/>
+      <c r="B139" s="15"/>
+      <c r="C139" s="15"/>
+      <c r="D139" s="15"/>
+      <c r="E139" s="15"/>
+      <c r="F139" s="15"/>
+      <c r="G139" s="15"/>
+      <c r="H139" s="15"/>
       <c r="I139" s="8">
         <v>0.11</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A140" s="13" t="s">
+    <row r="140" spans="1:9" ht="18" customHeight="1">
+      <c r="A140" s="12" t="s">
         <v>257</v>
       </c>
-      <c r="B140" s="11"/>
-      <c r="C140" s="11"/>
-      <c r="D140" s="11"/>
-      <c r="E140" s="11"/>
-      <c r="F140" s="11"/>
-      <c r="G140" s="11"/>
-      <c r="H140" s="11"/>
+      <c r="B140" s="15"/>
+      <c r="C140" s="15"/>
+      <c r="D140" s="15"/>
+      <c r="E140" s="15"/>
+      <c r="F140" s="15"/>
+      <c r="G140" s="15"/>
+      <c r="H140" s="15"/>
       <c r="I140" s="6">
         <v>1.8</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:9" ht="24" customHeight="1">
       <c r="A142" s="2" t="s">
         <v>140</v>
       </c>
@@ -5318,67 +5312,67 @@
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A143" s="14" t="s">
+    <row r="143" spans="1:9" ht="15" customHeight="1">
+      <c r="A143" s="13" t="s">
         <v>258</v>
       </c>
-      <c r="B143" s="11"/>
-      <c r="C143" s="11"/>
-      <c r="D143" s="11"/>
-      <c r="E143" s="11"/>
-      <c r="F143" s="11"/>
-      <c r="G143" s="11"/>
-      <c r="H143" s="11"/>
+      <c r="B143" s="15"/>
+      <c r="C143" s="15"/>
+      <c r="D143" s="15"/>
+      <c r="E143" s="15"/>
+      <c r="F143" s="15"/>
+      <c r="G143" s="15"/>
+      <c r="H143" s="15"/>
       <c r="I143" s="8">
         <v>2.2200000000000002</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A144" s="14" t="s">
+    <row r="144" spans="1:9" ht="15" customHeight="1">
+      <c r="A144" s="13" t="s">
         <v>259</v>
       </c>
-      <c r="B144" s="11"/>
-      <c r="C144" s="11"/>
-      <c r="D144" s="11"/>
-      <c r="E144" s="11"/>
-      <c r="F144" s="11"/>
-      <c r="G144" s="11"/>
-      <c r="H144" s="11"/>
+      <c r="B144" s="15"/>
+      <c r="C144" s="15"/>
+      <c r="D144" s="15"/>
+      <c r="E144" s="15"/>
+      <c r="F144" s="15"/>
+      <c r="G144" s="15"/>
+      <c r="H144" s="15"/>
       <c r="I144" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A145" s="14" t="s">
+    <row r="145" spans="1:9" ht="15" customHeight="1">
+      <c r="A145" s="13" t="s">
         <v>260</v>
       </c>
-      <c r="B145" s="11"/>
-      <c r="C145" s="11"/>
-      <c r="D145" s="11"/>
-      <c r="E145" s="11"/>
-      <c r="F145" s="11"/>
-      <c r="G145" s="11"/>
-      <c r="H145" s="11"/>
+      <c r="B145" s="15"/>
+      <c r="C145" s="15"/>
+      <c r="D145" s="15"/>
+      <c r="E145" s="15"/>
+      <c r="F145" s="15"/>
+      <c r="G145" s="15"/>
+      <c r="H145" s="15"/>
       <c r="I145" s="8">
         <v>0.15</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A146" s="13" t="s">
+    <row r="146" spans="1:9" ht="18" customHeight="1">
+      <c r="A146" s="12" t="s">
         <v>261</v>
       </c>
-      <c r="B146" s="11"/>
-      <c r="C146" s="11"/>
-      <c r="D146" s="11"/>
-      <c r="E146" s="11"/>
-      <c r="F146" s="11"/>
-      <c r="G146" s="11"/>
-      <c r="H146" s="11"/>
+      <c r="B146" s="15"/>
+      <c r="C146" s="15"/>
+      <c r="D146" s="15"/>
+      <c r="E146" s="15"/>
+      <c r="F146" s="15"/>
+      <c r="G146" s="15"/>
+      <c r="H146" s="15"/>
       <c r="I146" s="6">
         <v>2.37</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:9" ht="24" customHeight="1">
       <c r="A148" s="2" t="s">
         <v>144</v>
       </c>
@@ -5407,67 +5401,67 @@
         <v>13.62</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A149" s="14" t="s">
+    <row r="149" spans="1:9" ht="15" customHeight="1">
+      <c r="A149" s="13" t="s">
         <v>262</v>
       </c>
-      <c r="B149" s="11"/>
-      <c r="C149" s="11"/>
-      <c r="D149" s="11"/>
-      <c r="E149" s="11"/>
-      <c r="F149" s="11"/>
-      <c r="G149" s="11"/>
-      <c r="H149" s="11"/>
+      <c r="B149" s="15"/>
+      <c r="C149" s="15"/>
+      <c r="D149" s="15"/>
+      <c r="E149" s="15"/>
+      <c r="F149" s="15"/>
+      <c r="G149" s="15"/>
+      <c r="H149" s="15"/>
       <c r="I149" s="8">
         <v>13.62</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A150" s="14" t="s">
+    <row r="150" spans="1:9" ht="15" customHeight="1">
+      <c r="A150" s="13" t="s">
         <v>263</v>
       </c>
-      <c r="B150" s="11"/>
-      <c r="C150" s="11"/>
-      <c r="D150" s="11"/>
-      <c r="E150" s="11"/>
-      <c r="F150" s="11"/>
-      <c r="G150" s="11"/>
-      <c r="H150" s="11"/>
+      <c r="B150" s="15"/>
+      <c r="C150" s="15"/>
+      <c r="D150" s="15"/>
+      <c r="E150" s="15"/>
+      <c r="F150" s="15"/>
+      <c r="G150" s="15"/>
+      <c r="H150" s="15"/>
       <c r="I150" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A151" s="14" t="s">
+    <row r="151" spans="1:9" ht="15" customHeight="1">
+      <c r="A151" s="13" t="s">
         <v>264</v>
       </c>
-      <c r="B151" s="11"/>
-      <c r="C151" s="11"/>
-      <c r="D151" s="11"/>
-      <c r="E151" s="11"/>
-      <c r="F151" s="11"/>
-      <c r="G151" s="11"/>
-      <c r="H151" s="11"/>
+      <c r="B151" s="15"/>
+      <c r="C151" s="15"/>
+      <c r="D151" s="15"/>
+      <c r="E151" s="15"/>
+      <c r="F151" s="15"/>
+      <c r="G151" s="15"/>
+      <c r="H151" s="15"/>
       <c r="I151" s="8">
         <v>0.9</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A152" s="13" t="s">
+    <row r="152" spans="1:9" ht="18" customHeight="1">
+      <c r="A152" s="12" t="s">
         <v>265</v>
       </c>
-      <c r="B152" s="11"/>
-      <c r="C152" s="11"/>
-      <c r="D152" s="11"/>
-      <c r="E152" s="11"/>
-      <c r="F152" s="11"/>
-      <c r="G152" s="11"/>
-      <c r="H152" s="11"/>
+      <c r="B152" s="15"/>
+      <c r="C152" s="15"/>
+      <c r="D152" s="15"/>
+      <c r="E152" s="15"/>
+      <c r="F152" s="15"/>
+      <c r="G152" s="15"/>
+      <c r="H152" s="15"/>
       <c r="I152" s="6">
         <v>14.52</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:9" ht="24" customHeight="1">
       <c r="A154" s="2" t="s">
         <v>148</v>
       </c>
@@ -5496,122 +5490,122 @@
         <v>3.29</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A155" s="14" t="s">
+    <row r="155" spans="1:9" ht="15" customHeight="1">
+      <c r="A155" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="B155" s="11"/>
-      <c r="C155" s="11"/>
-      <c r="D155" s="11"/>
-      <c r="E155" s="11"/>
-      <c r="F155" s="11"/>
-      <c r="G155" s="11"/>
-      <c r="H155" s="11"/>
+      <c r="B155" s="15"/>
+      <c r="C155" s="15"/>
+      <c r="D155" s="15"/>
+      <c r="E155" s="15"/>
+      <c r="F155" s="15"/>
+      <c r="G155" s="15"/>
+      <c r="H155" s="15"/>
       <c r="I155" s="8">
         <v>3.29</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A156" s="14" t="s">
+    <row r="156" spans="1:9" ht="15" customHeight="1">
+      <c r="A156" s="13" t="s">
         <v>267</v>
       </c>
-      <c r="B156" s="11"/>
-      <c r="C156" s="11"/>
-      <c r="D156" s="11"/>
-      <c r="E156" s="11"/>
-      <c r="F156" s="11"/>
-      <c r="G156" s="11"/>
-      <c r="H156" s="11"/>
+      <c r="B156" s="15"/>
+      <c r="C156" s="15"/>
+      <c r="D156" s="15"/>
+      <c r="E156" s="15"/>
+      <c r="F156" s="15"/>
+      <c r="G156" s="15"/>
+      <c r="H156" s="15"/>
       <c r="I156" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A157" s="14" t="s">
+    <row r="157" spans="1:9" ht="15" customHeight="1">
+      <c r="A157" s="13" t="s">
         <v>268</v>
       </c>
-      <c r="B157" s="11"/>
-      <c r="C157" s="11"/>
-      <c r="D157" s="11"/>
-      <c r="E157" s="11"/>
-      <c r="F157" s="11"/>
-      <c r="G157" s="11"/>
-      <c r="H157" s="11"/>
+      <c r="B157" s="15"/>
+      <c r="C157" s="15"/>
+      <c r="D157" s="15"/>
+      <c r="E157" s="15"/>
+      <c r="F157" s="15"/>
+      <c r="G157" s="15"/>
+      <c r="H157" s="15"/>
       <c r="I157" s="8">
         <v>0.22</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A158" s="13" t="s">
+    <row r="158" spans="1:9" ht="18" customHeight="1">
+      <c r="A158" s="12" t="s">
         <v>269</v>
       </c>
-      <c r="B158" s="11"/>
-      <c r="C158" s="11"/>
-      <c r="D158" s="11"/>
-      <c r="E158" s="11"/>
-      <c r="F158" s="11"/>
-      <c r="G158" s="11"/>
-      <c r="H158" s="11"/>
+      <c r="B158" s="15"/>
+      <c r="C158" s="15"/>
+      <c r="D158" s="15"/>
+      <c r="E158" s="15"/>
+      <c r="F158" s="15"/>
+      <c r="G158" s="15"/>
+      <c r="H158" s="15"/>
       <c r="I158" s="6">
         <v>3.51</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A160" s="14" t="s">
+    <row r="160" spans="1:9" ht="15" customHeight="1">
+      <c r="A160" s="13" t="s">
         <v>270</v>
       </c>
-      <c r="B160" s="11"/>
-      <c r="C160" s="11"/>
-      <c r="D160" s="11"/>
-      <c r="E160" s="11"/>
-      <c r="F160" s="11"/>
-      <c r="G160" s="11"/>
-      <c r="H160" s="11"/>
+      <c r="B160" s="15"/>
+      <c r="C160" s="15"/>
+      <c r="D160" s="15"/>
+      <c r="E160" s="15"/>
+      <c r="F160" s="15"/>
+      <c r="G160" s="15"/>
+      <c r="H160" s="15"/>
       <c r="I160" s="8">
         <v>155.13999999999999</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A161" s="14" t="s">
+    <row r="161" spans="1:9" ht="15" customHeight="1">
+      <c r="A161" s="13" t="s">
         <v>271</v>
       </c>
-      <c r="B161" s="11"/>
-      <c r="C161" s="11"/>
-      <c r="D161" s="11"/>
-      <c r="E161" s="11"/>
-      <c r="F161" s="11"/>
-      <c r="G161" s="11"/>
-      <c r="H161" s="11"/>
+      <c r="B161" s="15"/>
+      <c r="C161" s="15"/>
+      <c r="D161" s="15"/>
+      <c r="E161" s="15"/>
+      <c r="F161" s="15"/>
+      <c r="G161" s="15"/>
+      <c r="H161" s="15"/>
       <c r="I161" s="8">
         <v>8.27</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A162" s="14" t="s">
+    <row r="162" spans="1:9" ht="15" customHeight="1">
+      <c r="A162" s="13" t="s">
         <v>272</v>
       </c>
-      <c r="B162" s="11"/>
-      <c r="C162" s="11"/>
-      <c r="D162" s="11"/>
-      <c r="E162" s="11"/>
-      <c r="F162" s="11"/>
-      <c r="G162" s="11"/>
-      <c r="H162" s="11"/>
+      <c r="B162" s="15"/>
+      <c r="C162" s="15"/>
+      <c r="D162" s="15"/>
+      <c r="E162" s="15"/>
+      <c r="F162" s="15"/>
+      <c r="G162" s="15"/>
+      <c r="H162" s="15"/>
       <c r="I162" s="8">
         <v>11.09</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A163" s="13" t="s">
+    <row r="163" spans="1:9" ht="18" customHeight="1">
+      <c r="A163" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="B163" s="11"/>
-      <c r="C163" s="11"/>
-      <c r="D163" s="11"/>
-      <c r="E163" s="11"/>
-      <c r="F163" s="11"/>
-      <c r="G163" s="11"/>
-      <c r="H163" s="11"/>
+      <c r="B163" s="15"/>
+      <c r="C163" s="15"/>
+      <c r="D163" s="15"/>
+      <c r="E163" s="15"/>
+      <c r="F163" s="15"/>
+      <c r="G163" s="15"/>
+      <c r="H163" s="15"/>
       <c r="I163" s="6">
         <v>174.5</v>
       </c>
@@ -5735,7 +5729,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -5746,18 +5740,18 @@
     <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:7" ht="27.95" customHeight="1">
+      <c r="A1" s="11" t="s">
         <v>274</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-    </row>
-    <row r="2" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+    </row>
+    <row r="2" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>165</v>
       </c>
@@ -5780,7 +5774,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="26.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>27</v>
       </c>
@@ -5803,7 +5797,7 @@
         <v>6.49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="26.1" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>33</v>
       </c>
@@ -5826,7 +5820,7 @@
         <v>37.99</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="26.1" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>37</v>
       </c>
@@ -5849,7 +5843,7 @@
         <v>59.99</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="26.1" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
@@ -5872,7 +5866,7 @@
         <v>14.39</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="26.1" customHeight="1">
       <c r="A7" s="2" t="s">
         <v>43</v>
       </c>
@@ -5895,54 +5889,54 @@
         <v>14.39</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
+    <row r="8" spans="1:7" ht="18" customHeight="1">
+      <c r="A8" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
       <c r="G8" s="9">
         <v>133.25</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:7" ht="18" customHeight="1">
+      <c r="A9" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
       <c r="G9" s="9">
         <v>6.99</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="15" t="s">
+    <row r="10" spans="1:7" ht="18" customHeight="1">
+      <c r="A10" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="9">
         <v>9.2799999999999994</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:7" ht="18" customHeight="1">
+      <c r="A11" s="12" t="s">
         <v>277</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="11"/>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="15"/>
       <c r="G11" s="6">
         <v>149.52000000000001</v>
       </c>
@@ -5962,7 +5956,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
     <col min="2" max="2" width="32" customWidth="1"/>
@@ -5973,18 +5967,18 @@
     <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="28" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:7" ht="27.95" customHeight="1">
+      <c r="A1" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-    </row>
-    <row r="2" spans="1:7" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+    </row>
+    <row r="2" spans="1:7" ht="20.100000000000001" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>165</v>
       </c>
@@ -6007,7 +6001,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="26.1" customHeight="1">
       <c r="A3" s="2" t="s">
         <v>150</v>
       </c>
@@ -6030,7 +6024,7 @@
         <v>8.99</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="26.1" customHeight="1">
       <c r="A4" s="2" t="s">
         <v>154</v>
       </c>
@@ -6053,7 +6047,7 @@
         <v>26.97</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="26.1" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>157</v>
       </c>
@@ -6076,7 +6070,7 @@
         <v>7.99</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="26.1" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>160</v>
       </c>
@@ -6099,54 +6093,54 @@
         <v>7.99</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+    <row r="7" spans="1:7" ht="18" customHeight="1">
+      <c r="A7" s="14" t="s">
         <v>276</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="11"/>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15"/>
       <c r="G7" s="9">
         <v>51.94</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="15" t="s">
+    <row r="8" spans="1:7" ht="18" customHeight="1">
+      <c r="A8" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
       <c r="G8" s="9">
         <v>6.99</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:7" ht="18" customHeight="1">
+      <c r="A9" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
       <c r="G9" s="9">
         <v>3.94</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="13" t="s">
+    <row r="10" spans="1:7" ht="18" customHeight="1">
+      <c r="A10" s="12" t="s">
         <v>277</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
       <c r="G10" s="6">
         <v>62.87</v>
       </c>

</xml_diff>